<commit_message>
actualizacion para el reporte fism segunda parte
</commit_message>
<xml_diff>
--- a/Ceduver/Uploads/Ficha/FISMNEW.xlsx
+++ b/Ceduver/Uploads/Ficha/FISMNEW.xlsx
@@ -66,7 +66,7 @@
     <t>MES:</t>
   </si>
   <si>
-    <t>septiembre</t>
+    <t>octubre</t>
   </si>
   <si>
     <t>DATOS GENERALES</t>
@@ -117,13 +117,13 @@
     <t>SALDO</t>
   </si>
   <si>
-    <t>FUENTE DE FINANCIAMIENTO: $0.00</t>
+    <t>FUENTE DE FINANCIAMIENTO: $22,222.00</t>
   </si>
   <si>
     <t>FUENTE DE FINANCIAMIENTO</t>
   </si>
   <si>
-    <t>TOTAL: $0.00</t>
+    <t>TOTAL: $22,222.00</t>
   </si>
   <si>
     <t>TOTAL</t>
@@ -171,7 +171,7 @@
     <t>NO. CONTRATO</t>
   </si>
   <si>
-    <t>01/01/1900</t>
+    <t>16/01/2023</t>
   </si>
   <si>
     <t>16/02/2023</t>
@@ -3333,7 +3333,7 @@
         <v>26</v>
       </c>
       <c r="F19" s="192">
-        <v>-36524.25</v>
+        <v>-14302.25</v>
       </c>
     </row>
     <row r="20" ht="23.25" customHeight="1">
@@ -3352,7 +3352,7 @@
         <v>28</v>
       </c>
       <c r="F20" s="217">
-        <v>-36524.25</v>
+        <v>-14302.25</v>
       </c>
     </row>
     <row r="21" ht="16.5" customHeight="1">

</xml_diff>

<commit_message>
REFINANDO PROBLEMA DE PERDIDA DE DATOS EN SEGUIMIENTO Y FINAL
</commit_message>
<xml_diff>
--- a/Ceduver/Uploads/Ficha/FISMNEW.xlsx
+++ b/Ceduver/Uploads/Ficha/FISMNEW.xlsx
@@ -117,13 +117,13 @@
     <t>SALDO</t>
   </si>
   <si>
-    <t>FUENTE DE FINANCIAMIENTO: $22,222.00</t>
+    <t>FUENTE DE FINANCIAMIENTO: $0.00</t>
   </si>
   <si>
     <t>FUENTE DE FINANCIAMIENTO</t>
   </si>
   <si>
-    <t>TOTAL: $22,222.00</t>
+    <t>TOTAL: $0.00</t>
   </si>
   <si>
     <t>TOTAL</t>
@@ -171,7 +171,7 @@
     <t>NO. CONTRATO</t>
   </si>
   <si>
-    <t>16/01/2023</t>
+    <t>01/01/1900</t>
   </si>
   <si>
     <t>16/02/2023</t>
@@ -3333,7 +3333,7 @@
         <v>26</v>
       </c>
       <c r="F19" s="192">
-        <v>-14302.25</v>
+        <v>-36524.25</v>
       </c>
     </row>
     <row r="20" ht="23.25" customHeight="1">
@@ -3352,7 +3352,7 @@
         <v>28</v>
       </c>
       <c r="F20" s="217">
-        <v>-14302.25</v>
+        <v>-36524.25</v>
       </c>
     </row>
     <row r="21" ht="16.5" customHeight="1">

</xml_diff>